<commit_message>
feat: pushing the final code
</commit_message>
<xml_diff>
--- a/synthetic_data/exhibit3.xlsx
+++ b/synthetic_data/exhibit3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exhibit 3" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Exhibit 3" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -111,11 +111,88 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,6 +220,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -587,6 +667,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -605,25 +686,25 @@
           <t>Module 1</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="14" t="n"/>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Module 2</t>
         </is>
       </c>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="14" t="n"/>
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Module 3</t>
         </is>
       </c>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
+      <c r="A6" s="15" t="n"/>
       <c r="B6" s="7" t="inlineStr">
         <is>
           <t>A</t>
@@ -688,29 +769,65 @@
       <c r="A8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
+      <c r="B8" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
+      <c r="B9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -779,9 +896,9 @@
   <mergeCells count="8">
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B5:D5"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="H5:J5"/>

</xml_diff>